<commit_message>
docs(roadmap): aggiornato Step.md con tabella riassuntiva GUI, ipertesti Excel e post-fetch filter MAUDE
</commit_message>
<xml_diff>
--- a/PMS_Report_DPR-385_Period_2025-07-26_to_2026-07-26.xlsx
+++ b/PMS_Report_DPR-385_Period_2025-07-26_to_2026-07-26.xlsx
@@ -472,7 +472,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>This document serves as a worksheet for collecting vigilance data from the main DB for the PMS of mammography, web based viewer.</t>
+          <t>This document serves as a worksheet for collecting vigilance data from the main DB for the PMS of DICOM viewer.</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Period 2025-07-26 to 2026-07-26</t>
+          <t>2025-07-26 to 2026-07-26</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-07-26 16:39</t>
+          <t>2026-07-26 17:23</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -612,7 +612,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>"mammography"</t>
+          <t>"DICOM viewer"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -719,7 +719,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -812,214 +812,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>"web based viewer"</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Tot:</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Tot:</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Tot:</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Tot:</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Tot:</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Tot:</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Tot:</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Tot:</t>
-        </is>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Dupl:</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Dupl:</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Dupl:</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Dupl:</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Dupl:</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Dupl:</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Dupl:</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Dupl:</t>
-        </is>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Sel:</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Sel:</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Sel:</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Sel:</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Sel:</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Sel:</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Sel:</t>
-        </is>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>Sel:</t>
-        </is>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="10">
     <mergeCell ref="Q1:R1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="A2:A4"/>
@@ -1027,11 +821,9 @@
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="O1:P1"/>
-    <mergeCell ref="A5:A7"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="B5:B7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>